<commit_message>
docs(hubs): update hub BRDs, vehicle car model detail PRD, and September 2026 performance reports
</commit_message>
<xml_diff>
--- a/05_HUBS/cinema/cinema-hub-roadmap.xlsx
+++ b/05_HUBS/cinema/cinema-hub-roadmap.xlsx
@@ -2400,21 +2400,21 @@
   <dimension ref="A1:Y1017"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="31" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
     <col width="23" customWidth="1" min="3" max="3"/>
     <col width="29" customWidth="1" min="4" max="4"/>
     <col width="25" customWidth="1" min="5" max="5"/>
     <col width="23" customWidth="1" min="6" max="6"/>
     <col width="23" customWidth="1" min="7" max="7"/>
-    <col width="67" customWidth="1" min="8" max="8"/>
+    <col width="84" customWidth="1" min="8" max="8"/>
     <col width="14" customWidth="1" min="9" max="9"/>
     <col width="23" customWidth="1" min="10" max="10"/>
     <col width="23" customWidth="1" min="11" max="11"/>
     <col width="23" customWidth="1" min="12" max="12"/>
     <col width="23" customWidth="1" min="13" max="13"/>
     <col width="23" customWidth="1" min="14" max="14"/>
-    <col width="16" customWidth="1" min="15" max="15"/>
+    <col width="15" customWidth="1" min="15" max="15"/>
     <col width="23" customWidth="1" min="16" max="16"/>
     <col width="23" customWidth="1" min="17" max="17"/>
     <col width="23" customWidth="1" min="18" max="18"/>
@@ -2430,14 +2430,14 @@
     <row r="1">
       <c r="A1" s="6" t="inlineStr">
         <is>
-          <t>BÁO CÁO PHÂN TÍCH HIỆU SUẤT VẬN HÀNH &amp; TRAFFIC - CINEMA HUB (MTD 26D - CẮT NGÀY 26/09/2026)</t>
+          <t>BÁO CÁO PHÂN TÍCH HIỆU SUẤT VẬN HÀNH &amp; TRAFFIC - CINEMA HUB (MTD 27D - CẮT NGÀY 27/09/2026)</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="49" t="inlineStr">
         <is>
-          <t>Nguồn dữ liệu Single Source of Truth (SSOT): /Users/hienhv/Downloads/Web Performance Tracking (1).xlsx</t>
+          <t>Nguồn dữ liệu Single Source of Truth (SSOT): /Users/hienhv/Downloads/Web Performance Tracking.xlsx</t>
         </is>
       </c>
     </row>
@@ -2455,7 +2455,7 @@
       </c>
       <c r="C4" s="50" t="inlineStr">
         <is>
-          <t>Số Thực Tế MTD 26d</t>
+          <t>Số Thực Tế MTD 27d</t>
         </is>
       </c>
       <c r="D4" s="50" t="inlineStr">
@@ -2496,23 +2496,23 @@
         </is>
       </c>
       <c r="C5" s="52" t="n">
-        <v>1033573</v>
+        <v>1086874</v>
       </c>
       <c r="D5" s="52" t="n">
-        <v>39752.8</v>
+        <v>40254.6</v>
       </c>
       <c r="E5" s="52" t="n">
-        <v>1192584.2</v>
+        <v>1207637.8</v>
       </c>
       <c r="F5" s="52" t="n">
         <v>1500000</v>
       </c>
       <c r="G5" s="53" t="n">
-        <v>0.7951</v>
+        <v>0.8051</v>
       </c>
       <c r="H5" s="51" t="inlineStr">
         <is>
-          <t>CHÍNH THỨC VƯỢT MỐC LỊCH SỬ &gt;1 TRIỆU PVS MTD (79.5% Target Hub)</t>
+          <t>CÁN MỐC LỊCH SỬ &gt;1.08 TRIỆU PVS MTD (80.5% Target Hub, Forecast trọn tháng 1.2M)</t>
         </is>
       </c>
     </row>
@@ -2520,7 +2520,7 @@
     <row r="7" ht="26" customHeight="1">
       <c r="A7" s="6" t="inlineStr">
         <is>
-          <t>CHI TIẾT LƯU LƯỢNG TRUY CẬP LỊCH SỬ THEO DỰ ÁN &amp; KÊNH TRAFFIC (THÁNG 5 -&gt; THÁNG 9 MTD 26D)</t>
+          <t>CHI TIẾT LƯU LƯỢNG TRUY CẬP LỊCH SỬ THEO DỰ ÁN &amp; KÊNH TRAFFIC (THÁNG 5 -&gt; THÁNG 9 MTD 27D)</t>
         </is>
       </c>
     </row>
@@ -2533,7 +2533,7 @@
       </c>
       <c r="B9" s="54" t="inlineStr">
         <is>
-          <t>MTD</t>
+          <t>Update to: 26</t>
         </is>
       </c>
       <c r="C9" s="55" t="n">
@@ -2601,55 +2601,37 @@
     <row r="10" ht="26" customHeight="1">
       <c r="A10" s="56" t="inlineStr">
         <is>
-          <t>Traffic Actual (Page Views)</t>
+          <t xml:space="preserve">   Target</t>
         </is>
       </c>
       <c r="B10" s="56" t="n"/>
-      <c r="C10" s="52" t="n">
-        <v>888178</v>
-      </c>
-      <c r="D10" s="52" t="n">
-        <v>780270</v>
-      </c>
-      <c r="E10" s="52" t="n">
-        <v>720040</v>
-      </c>
-      <c r="F10" s="52" t="n">
-        <v>669345</v>
-      </c>
-      <c r="G10" s="52" t="n">
-        <v>1033573</v>
-      </c>
-      <c r="H10" s="52" t="n">
-        <v>364228</v>
-      </c>
+      <c r="C10" s="56" t="n"/>
+      <c r="D10" s="56" t="n"/>
+      <c r="E10" s="56" t="n"/>
+      <c r="F10" s="56" t="n"/>
+      <c r="G10" s="56" t="n"/>
+      <c r="H10" s="56" t="n"/>
       <c r="I10" s="56" t="n"/>
-      <c r="J10" s="52" t="n">
-        <v>994719</v>
-      </c>
-      <c r="K10" s="52" t="n">
-        <v>859183</v>
-      </c>
+      <c r="J10" s="56" t="n"/>
+      <c r="K10" s="56" t="n"/>
       <c r="L10" s="52" t="n">
-        <v>822859</v>
+        <v>0</v>
       </c>
       <c r="M10" s="52" t="n">
-        <v>832356</v>
+        <v>0</v>
       </c>
       <c r="N10" s="52" t="n">
-        <v>1033573</v>
-      </c>
-      <c r="O10" s="52" t="n">
-        <v>201217</v>
-      </c>
+        <v>964394.3350400146</v>
+      </c>
+      <c r="O10" s="56" t="n"/>
       <c r="P10" s="52" t="n">
-        <v>0</v>
+        <v>1117378.181279731</v>
       </c>
       <c r="Q10" s="52" t="n">
-        <v>0</v>
+        <v>1294630.168009226</v>
       </c>
       <c r="R10" s="52" t="n">
-        <v>0</v>
+        <v>1500000</v>
       </c>
       <c r="S10" s="56" t="n"/>
       <c r="T10" s="56" t="n"/>
@@ -2662,37 +2644,55 @@
     <row r="11" ht="26" customHeight="1">
       <c r="A11" s="57" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Target</t>
+          <t xml:space="preserve">   Traffic Actual (Page Views)</t>
         </is>
       </c>
       <c r="B11" s="57" t="n"/>
-      <c r="C11" s="57" t="n"/>
-      <c r="D11" s="57" t="n"/>
-      <c r="E11" s="57" t="n"/>
-      <c r="F11" s="57" t="n"/>
-      <c r="G11" s="57" t="n"/>
-      <c r="H11" s="57" t="n"/>
+      <c r="C11" s="58" t="n">
+        <v>912528</v>
+      </c>
+      <c r="D11" s="58" t="n">
+        <v>808378</v>
+      </c>
+      <c r="E11" s="58" t="n">
+        <v>742783</v>
+      </c>
+      <c r="F11" s="58" t="n">
+        <v>699471</v>
+      </c>
+      <c r="G11" s="58" t="n">
+        <v>1086874</v>
+      </c>
+      <c r="H11" s="58" t="n">
+        <v>387403</v>
+      </c>
       <c r="I11" s="57" t="n"/>
-      <c r="J11" s="57" t="n"/>
-      <c r="K11" s="57" t="n"/>
+      <c r="J11" s="58" t="n">
+        <v>994719</v>
+      </c>
+      <c r="K11" s="58" t="n">
+        <v>859183</v>
+      </c>
       <c r="L11" s="58" t="n">
+        <v>822859</v>
+      </c>
+      <c r="M11" s="57" t="n">
+        <v>832356</v>
+      </c>
+      <c r="N11" s="57" t="n">
+        <v>1086874</v>
+      </c>
+      <c r="O11" s="57" t="n">
+        <v>254518</v>
+      </c>
+      <c r="P11" s="57" t="n">
         <v>0</v>
       </c>
-      <c r="M11" s="57" t="n">
+      <c r="Q11" s="57" t="n">
         <v>0</v>
       </c>
-      <c r="N11" s="57" t="n">
-        <v>964394.3350400146</v>
-      </c>
-      <c r="O11" s="57" t="n"/>
-      <c r="P11" s="57" t="n">
-        <v>1117378.181279731</v>
-      </c>
-      <c r="Q11" s="57" t="n">
-        <v>1294630.168009226</v>
-      </c>
       <c r="R11" s="57" t="n">
-        <v>1500000</v>
+        <v>0</v>
       </c>
       <c r="S11" s="57" t="n"/>
       <c r="T11" s="57" t="n"/>
@@ -2710,19 +2710,19 @@
       </c>
       <c r="B12" s="57" t="n"/>
       <c r="C12" s="58" t="n">
-        <v>888178</v>
+        <v>912528</v>
       </c>
       <c r="D12" s="58" t="n">
-        <v>-107908</v>
+        <v>-104150</v>
       </c>
       <c r="E12" s="58" t="n">
-        <v>-60230</v>
+        <v>-65595</v>
       </c>
       <c r="F12" s="58" t="n">
-        <v>-50695</v>
+        <v>-43312</v>
       </c>
       <c r="G12" s="58" t="n">
-        <v>364228</v>
+        <v>387403</v>
       </c>
       <c r="H12" s="57" t="n"/>
       <c r="I12" s="57" t="n"/>
@@ -2739,7 +2739,7 @@
         <v>9497</v>
       </c>
       <c r="N12" s="57" t="n">
-        <v>201217</v>
+        <v>254518</v>
       </c>
       <c r="O12" s="57" t="n"/>
       <c r="P12" s="57" t="n">
@@ -2768,19 +2768,19 @@
       <c r="B13" s="57" t="n"/>
       <c r="C13" s="57" t="n"/>
       <c r="D13" s="58" t="n">
-        <v>-0.1214936646</v>
+        <v>-0.1141334841</v>
       </c>
       <c r="E13" s="58" t="n">
-        <v>-0.07719122868</v>
+        <v>-0.08114396978000001</v>
       </c>
       <c r="F13" s="58" t="n">
-        <v>-0.07040581079</v>
+        <v>-0.05831043521</v>
       </c>
       <c r="G13" s="58" t="n">
-        <v>0.5441558539</v>
+        <v>0.5538514106</v>
       </c>
       <c r="H13" s="58" t="n">
-        <v>0.6145616645999999</v>
+        <v>0.6121618458</v>
       </c>
       <c r="I13" s="57" t="n"/>
       <c r="J13" s="57" t="n"/>
@@ -2794,10 +2794,10 @@
         <v>0.01154146701</v>
       </c>
       <c r="N13" s="57" t="n">
-        <v>0.2417439173</v>
+        <v>0.305780219</v>
       </c>
       <c r="O13" s="57" t="n">
-        <v>0.2302024503</v>
+        <v>0.294238752</v>
       </c>
       <c r="P13" s="57" t="n">
         <v>0.1586320457</v>
@@ -2866,7 +2866,7 @@
       <c r="L15" s="57" t="n"/>
       <c r="M15" s="57" t="n"/>
       <c r="N15" s="57" t="n">
-        <v>69178.66495999999</v>
+        <v>122479.665</v>
       </c>
       <c r="O15" s="57" t="n"/>
       <c r="P15" s="57" t="n"/>
@@ -2915,22 +2915,22 @@
       </c>
       <c r="B17" s="57" t="n"/>
       <c r="C17" s="58" t="n">
-        <v>324827</v>
+        <v>336155</v>
       </c>
       <c r="D17" s="58" t="n">
-        <v>363635</v>
+        <v>377417</v>
       </c>
       <c r="E17" s="58" t="n">
-        <v>358182</v>
+        <v>369741</v>
       </c>
       <c r="F17" s="58" t="n">
-        <v>339600</v>
+        <v>354449</v>
       </c>
       <c r="G17" s="58" t="n">
-        <v>376365</v>
+        <v>411613</v>
       </c>
       <c r="H17" s="58" t="n">
-        <v>36765</v>
+        <v>57164</v>
       </c>
       <c r="I17" s="57" t="n"/>
       <c r="J17" s="58" t="n">
@@ -2946,10 +2946,10 @@
         <v>418684</v>
       </c>
       <c r="N17" s="57" t="n">
-        <v>376365</v>
+        <v>411613</v>
       </c>
       <c r="O17" s="57" t="n">
-        <v>-42319</v>
+        <v>-7071</v>
       </c>
       <c r="P17" s="57" t="n"/>
       <c r="Q17" s="57" t="n"/>
@@ -2970,22 +2970,22 @@
         </is>
       </c>
       <c r="C18" s="58" t="n">
-        <v>305523</v>
+        <v>316257</v>
       </c>
       <c r="D18" s="58" t="n">
-        <v>344554</v>
+        <v>357696</v>
       </c>
       <c r="E18" s="58" t="n">
-        <v>340713</v>
+        <v>351774</v>
       </c>
       <c r="F18" s="58" t="n">
-        <v>311512</v>
+        <v>324998</v>
       </c>
       <c r="G18" s="58" t="n">
-        <v>341868</v>
+        <v>376150</v>
       </c>
       <c r="H18" s="58" t="n">
-        <v>30356</v>
+        <v>51152</v>
       </c>
       <c r="I18" s="57" t="n"/>
       <c r="J18" s="58" t="n">
@@ -3001,10 +3001,10 @@
         <v>384126</v>
       </c>
       <c r="N18" s="57" t="n">
-        <v>341868</v>
+        <v>376150</v>
       </c>
       <c r="O18" s="57" t="n">
-        <v>-42258</v>
+        <v>-7976</v>
       </c>
       <c r="P18" s="57" t="n"/>
       <c r="Q18" s="57" t="n"/>
@@ -3025,22 +3025,22 @@
         </is>
       </c>
       <c r="C19" s="58" t="n">
-        <v>11168</v>
+        <v>11537</v>
       </c>
       <c r="D19" s="58" t="n">
-        <v>12530</v>
+        <v>12964</v>
       </c>
       <c r="E19" s="58" t="n">
-        <v>13270</v>
+        <v>13625</v>
       </c>
       <c r="F19" s="58" t="n">
-        <v>12193</v>
+        <v>12644</v>
       </c>
       <c r="G19" s="58" t="n">
-        <v>14509</v>
+        <v>15268</v>
       </c>
       <c r="H19" s="58" t="n">
-        <v>2316</v>
+        <v>2624</v>
       </c>
       <c r="I19" s="57" t="n"/>
       <c r="J19" s="58" t="n">
@@ -3056,10 +3056,10 @@
         <v>14529</v>
       </c>
       <c r="N19" s="57" t="n">
-        <v>14509</v>
+        <v>15268</v>
       </c>
       <c r="O19" s="57" t="n">
-        <v>-20</v>
+        <v>739</v>
       </c>
       <c r="P19" s="57" t="n"/>
       <c r="Q19" s="57" t="n"/>
@@ -3080,7 +3080,7 @@
         </is>
       </c>
       <c r="C20" s="58" t="n">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="D20" s="58" t="n">
         <v>116</v>
@@ -3089,13 +3089,13 @@
         <v>55</v>
       </c>
       <c r="F20" s="58" t="n">
-        <v>12183</v>
+        <v>12932</v>
       </c>
       <c r="G20" s="58" t="n">
-        <v>15700</v>
+        <v>15739</v>
       </c>
       <c r="H20" s="58" t="n">
-        <v>3517</v>
+        <v>2807</v>
       </c>
       <c r="I20" s="57" t="n"/>
       <c r="J20" s="58" t="n">
@@ -3111,10 +3111,10 @@
         <v>15523</v>
       </c>
       <c r="N20" s="57" t="n">
-        <v>15700</v>
+        <v>15739</v>
       </c>
       <c r="O20" s="57" t="n">
-        <v>177</v>
+        <v>216</v>
       </c>
       <c r="P20" s="57" t="n"/>
       <c r="Q20" s="57" t="n"/>
@@ -3135,22 +3135,22 @@
         </is>
       </c>
       <c r="C21" s="58" t="n">
-        <v>3207</v>
+        <v>3315</v>
       </c>
       <c r="D21" s="58" t="n">
-        <v>3827</v>
+        <v>3922</v>
       </c>
       <c r="E21" s="58" t="n">
-        <v>3532</v>
+        <v>3672</v>
       </c>
       <c r="F21" s="58" t="n">
-        <v>3397</v>
+        <v>3550</v>
       </c>
       <c r="G21" s="58" t="n">
-        <v>2790</v>
+        <v>2941</v>
       </c>
       <c r="H21" s="58" t="n">
-        <v>-607</v>
+        <v>-609</v>
       </c>
       <c r="I21" s="57" t="n"/>
       <c r="J21" s="58" t="n">
@@ -3166,10 +3166,10 @@
         <v>4095</v>
       </c>
       <c r="N21" s="57" t="n">
-        <v>2790</v>
+        <v>2941</v>
       </c>
       <c r="O21" s="57" t="n">
-        <v>-1305</v>
+        <v>-1154</v>
       </c>
       <c r="P21" s="57" t="n"/>
       <c r="Q21" s="57" t="n"/>
@@ -3190,22 +3190,22 @@
         </is>
       </c>
       <c r="C22" s="58" t="n">
-        <v>4825</v>
+        <v>4941</v>
       </c>
       <c r="D22" s="58" t="n">
-        <v>2608</v>
+        <v>2719</v>
       </c>
       <c r="E22" s="58" t="n">
-        <v>612</v>
+        <v>615</v>
       </c>
       <c r="F22" s="58" t="n">
-        <v>315</v>
+        <v>325</v>
       </c>
       <c r="G22" s="58" t="n">
-        <v>1498</v>
+        <v>1515</v>
       </c>
       <c r="H22" s="58" t="n">
-        <v>1183</v>
+        <v>1190</v>
       </c>
       <c r="I22" s="57" t="n"/>
       <c r="J22" s="58" t="n">
@@ -3221,10 +3221,10 @@
         <v>411</v>
       </c>
       <c r="N22" s="57" t="n">
-        <v>1498</v>
+        <v>1515</v>
       </c>
       <c r="O22" s="57" t="n">
-        <v>1087</v>
+        <v>1104</v>
       </c>
       <c r="P22" s="57" t="n"/>
       <c r="Q22" s="57" t="n"/>
@@ -3272,22 +3272,22 @@
       </c>
       <c r="B24" s="57" t="n"/>
       <c r="C24" s="58" t="n">
-        <v>466247</v>
+        <v>475523</v>
       </c>
       <c r="D24" s="58" t="n">
-        <v>320912</v>
+        <v>331789</v>
       </c>
       <c r="E24" s="58" t="n">
-        <v>274173</v>
+        <v>282300</v>
       </c>
       <c r="F24" s="58" t="n">
-        <v>252944</v>
+        <v>265373</v>
       </c>
       <c r="G24" s="58" t="n">
-        <v>593868</v>
+        <v>609544</v>
       </c>
       <c r="H24" s="58" t="n">
-        <v>340924</v>
+        <v>344171</v>
       </c>
       <c r="I24" s="57" t="n"/>
       <c r="J24" s="58" t="n">
@@ -3303,10 +3303,10 @@
         <v>324305</v>
       </c>
       <c r="N24" s="57" t="n">
-        <v>593868</v>
+        <v>609544</v>
       </c>
       <c r="O24" s="57" t="n">
-        <v>269563</v>
+        <v>285239</v>
       </c>
       <c r="P24" s="57" t="n"/>
       <c r="Q24" s="57" t="n"/>
@@ -3327,22 +3327,22 @@
         </is>
       </c>
       <c r="C25" s="58" t="n">
-        <v>257461</v>
+        <v>265457</v>
       </c>
       <c r="D25" s="58" t="n">
-        <v>244149</v>
+        <v>253062</v>
       </c>
       <c r="E25" s="58" t="n">
-        <v>227267</v>
+        <v>234285</v>
       </c>
       <c r="F25" s="58" t="n">
-        <v>213375</v>
+        <v>223970</v>
       </c>
       <c r="G25" s="58" t="n">
-        <v>233637</v>
+        <v>247366</v>
       </c>
       <c r="H25" s="58" t="n">
-        <v>20262</v>
+        <v>23396</v>
       </c>
       <c r="I25" s="57" t="n"/>
       <c r="J25" s="58" t="n">
@@ -3358,10 +3358,10 @@
         <v>265423</v>
       </c>
       <c r="N25" s="57" t="n">
-        <v>233637</v>
+        <v>247366</v>
       </c>
       <c r="O25" s="57" t="n">
-        <v>-31786</v>
+        <v>-18057</v>
       </c>
       <c r="P25" s="57" t="n"/>
       <c r="Q25" s="57" t="n"/>
@@ -3382,22 +3382,22 @@
         </is>
       </c>
       <c r="C26" s="58" t="n">
-        <v>192390</v>
+        <v>193112</v>
       </c>
       <c r="D26" s="58" t="n">
-        <v>38083</v>
+        <v>39744</v>
       </c>
       <c r="E26" s="58" t="n">
-        <v>35420</v>
+        <v>36309</v>
       </c>
       <c r="F26" s="58" t="n">
-        <v>25979</v>
+        <v>26996</v>
       </c>
       <c r="G26" s="58" t="n">
-        <v>21091</v>
+        <v>22325</v>
       </c>
       <c r="H26" s="58" t="n">
-        <v>-4888</v>
+        <v>-4671</v>
       </c>
       <c r="I26" s="57" t="n"/>
       <c r="J26" s="58" t="n">
@@ -3413,10 +3413,10 @@
         <v>30205</v>
       </c>
       <c r="N26" s="57" t="n">
-        <v>21091</v>
+        <v>22325</v>
       </c>
       <c r="O26" s="57" t="n">
-        <v>-9114</v>
+        <v>-7880</v>
       </c>
       <c r="P26" s="57" t="n"/>
       <c r="Q26" s="57" t="n"/>
@@ -3437,22 +3437,22 @@
         </is>
       </c>
       <c r="C27" s="58" t="n">
-        <v>992</v>
+        <v>1085</v>
       </c>
       <c r="D27" s="58" t="n">
-        <v>24228</v>
+        <v>24240</v>
       </c>
       <c r="E27" s="58" t="n">
-        <v>2083</v>
+        <v>2094</v>
       </c>
       <c r="F27" s="58" t="n">
-        <v>6332</v>
+        <v>6794</v>
       </c>
       <c r="G27" s="58" t="n">
-        <v>332181</v>
+        <v>332649</v>
       </c>
       <c r="H27" s="58" t="n">
-        <v>325849</v>
+        <v>325855</v>
       </c>
       <c r="I27" s="57" t="n"/>
       <c r="J27" s="58" t="n">
@@ -3468,10 +3468,10 @@
         <v>19946</v>
       </c>
       <c r="N27" s="57" t="n">
-        <v>332181</v>
+        <v>332649</v>
       </c>
       <c r="O27" s="57" t="n">
-        <v>312235</v>
+        <v>312703</v>
       </c>
       <c r="P27" s="57" t="n"/>
       <c r="Q27" s="57" t="n"/>
@@ -3492,22 +3492,22 @@
         </is>
       </c>
       <c r="C28" s="58" t="n">
-        <v>8342</v>
+        <v>8662</v>
       </c>
       <c r="D28" s="58" t="n">
-        <v>10770</v>
+        <v>10978</v>
       </c>
       <c r="E28" s="58" t="n">
-        <v>8476</v>
+        <v>8671</v>
       </c>
       <c r="F28" s="58" t="n">
-        <v>6554</v>
+        <v>6885</v>
       </c>
       <c r="G28" s="58" t="n">
-        <v>5514</v>
+        <v>5727</v>
       </c>
       <c r="H28" s="58" t="n">
-        <v>-1040</v>
+        <v>-1158</v>
       </c>
       <c r="I28" s="57" t="n"/>
       <c r="J28" s="58" t="n">
@@ -3523,10 +3523,10 @@
         <v>7898</v>
       </c>
       <c r="N28" s="57" t="n">
-        <v>5514</v>
+        <v>5727</v>
       </c>
       <c r="O28" s="57" t="n">
-        <v>-2384</v>
+        <v>-2171</v>
       </c>
       <c r="P28" s="57" t="n"/>
       <c r="Q28" s="57" t="n"/>
@@ -3547,22 +3547,22 @@
         </is>
       </c>
       <c r="C29" s="58" t="n">
-        <v>7062</v>
+        <v>7207</v>
       </c>
       <c r="D29" s="58" t="n">
-        <v>3682</v>
+        <v>3765</v>
       </c>
       <c r="E29" s="58" t="n">
-        <v>927</v>
+        <v>941</v>
       </c>
       <c r="F29" s="58" t="n">
-        <v>704</v>
+        <v>728</v>
       </c>
       <c r="G29" s="58" t="n">
-        <v>1445</v>
+        <v>1477</v>
       </c>
       <c r="H29" s="58" t="n">
-        <v>741</v>
+        <v>749</v>
       </c>
       <c r="I29" s="57" t="n"/>
       <c r="J29" s="58" t="n">
@@ -3578,10 +3578,10 @@
         <v>833</v>
       </c>
       <c r="N29" s="57" t="n">
-        <v>1445</v>
+        <v>1477</v>
       </c>
       <c r="O29" s="57" t="n">
-        <v>612</v>
+        <v>644</v>
       </c>
       <c r="P29" s="57" t="n"/>
       <c r="Q29" s="57" t="n"/>
@@ -3629,22 +3629,22 @@
       </c>
       <c r="B31" s="57" t="n"/>
       <c r="C31" s="58" t="n">
-        <v>65598</v>
+        <v>68257</v>
       </c>
       <c r="D31" s="58" t="n">
-        <v>60546</v>
+        <v>62748</v>
       </c>
       <c r="E31" s="58" t="n">
-        <v>49728</v>
+        <v>51627</v>
       </c>
       <c r="F31" s="58" t="n">
-        <v>44257</v>
+        <v>45830</v>
       </c>
       <c r="G31" s="58" t="n">
-        <v>37669</v>
+        <v>38594</v>
       </c>
       <c r="H31" s="58" t="n">
-        <v>-6588</v>
+        <v>-7236</v>
       </c>
       <c r="I31" s="57" t="n"/>
       <c r="J31" s="58" t="n">
@@ -3660,10 +3660,10 @@
         <v>51234</v>
       </c>
       <c r="N31" s="57" t="n">
-        <v>37669</v>
+        <v>38594</v>
       </c>
       <c r="O31" s="57" t="n">
-        <v>-13565</v>
+        <v>-12640</v>
       </c>
       <c r="P31" s="57" t="n"/>
       <c r="Q31" s="57" t="n"/>
@@ -3684,22 +3684,22 @@
         </is>
       </c>
       <c r="C32" s="58" t="n">
-        <v>58434</v>
+        <v>60812</v>
       </c>
       <c r="D32" s="58" t="n">
-        <v>53997</v>
+        <v>55958</v>
       </c>
       <c r="E32" s="58" t="n">
-        <v>43489</v>
+        <v>45188</v>
       </c>
       <c r="F32" s="58" t="n">
-        <v>38049</v>
+        <v>39413</v>
       </c>
       <c r="G32" s="58" t="n">
-        <v>32578</v>
+        <v>33345</v>
       </c>
       <c r="H32" s="58" t="n">
-        <v>-5471</v>
+        <v>-6068</v>
       </c>
       <c r="I32" s="57" t="n"/>
       <c r="J32" s="58" t="n">
@@ -3715,10 +3715,10 @@
         <v>44104</v>
       </c>
       <c r="N32" s="57" t="n">
-        <v>32578</v>
+        <v>33345</v>
       </c>
       <c r="O32" s="57" t="n">
-        <v>-11526</v>
+        <v>-10759</v>
       </c>
       <c r="P32" s="57" t="n"/>
       <c r="Q32" s="57" t="n"/>
@@ -3739,22 +3739,22 @@
         </is>
       </c>
       <c r="C33" s="58" t="n">
-        <v>3572</v>
+        <v>3704</v>
       </c>
       <c r="D33" s="58" t="n">
-        <v>3410</v>
+        <v>3520</v>
       </c>
       <c r="E33" s="58" t="n">
-        <v>3365</v>
+        <v>3482</v>
       </c>
       <c r="F33" s="58" t="n">
-        <v>2940</v>
+        <v>3027</v>
       </c>
       <c r="G33" s="58" t="n">
-        <v>2296</v>
+        <v>2381</v>
       </c>
       <c r="H33" s="58" t="n">
-        <v>-644</v>
+        <v>-646</v>
       </c>
       <c r="I33" s="57" t="n"/>
       <c r="J33" s="58" t="n">
@@ -3770,10 +3770,10 @@
         <v>3356</v>
       </c>
       <c r="N33" s="57" t="n">
-        <v>2296</v>
+        <v>2381</v>
       </c>
       <c r="O33" s="57" t="n">
-        <v>-1060</v>
+        <v>-975</v>
       </c>
       <c r="P33" s="57" t="n"/>
       <c r="Q33" s="57" t="n"/>
@@ -3794,22 +3794,22 @@
         </is>
       </c>
       <c r="C34" s="58" t="n">
-        <v>3198</v>
+        <v>3342</v>
       </c>
       <c r="D34" s="58" t="n">
-        <v>2992</v>
+        <v>3109</v>
       </c>
       <c r="E34" s="58" t="n">
-        <v>2807</v>
+        <v>2889</v>
       </c>
       <c r="F34" s="58" t="n">
-        <v>3140</v>
+        <v>3258</v>
       </c>
       <c r="G34" s="58" t="n">
-        <v>2472</v>
+        <v>2545</v>
       </c>
       <c r="H34" s="58" t="n">
-        <v>-668</v>
+        <v>-713</v>
       </c>
       <c r="I34" s="57" t="n"/>
       <c r="J34" s="58" t="n">
@@ -3825,10 +3825,10 @@
         <v>3634</v>
       </c>
       <c r="N34" s="57" t="n">
-        <v>2472</v>
+        <v>2545</v>
       </c>
       <c r="O34" s="57" t="n">
-        <v>-1162</v>
+        <v>-1089</v>
       </c>
       <c r="P34" s="57" t="n"/>
       <c r="Q34" s="57" t="n"/>
@@ -3849,22 +3849,22 @@
         </is>
       </c>
       <c r="C35" s="58" t="n">
-        <v>378</v>
+        <v>381</v>
       </c>
       <c r="D35" s="58" t="n">
-        <v>136</v>
+        <v>150</v>
       </c>
       <c r="E35" s="58" t="n">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="F35" s="58" t="n">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="G35" s="58" t="n">
         <v>159</v>
       </c>
       <c r="H35" s="58" t="n">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="I35" s="57" t="n"/>
       <c r="J35" s="58" t="n">
@@ -3904,7 +3904,7 @@
         </is>
       </c>
       <c r="C36" s="58" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="D36" s="58" t="n">
         <v>11</v>
@@ -3913,13 +3913,13 @@
         <v>3</v>
       </c>
       <c r="F36" s="58" t="n">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="G36" s="58" t="n">
         <v>164</v>
       </c>
       <c r="H36" s="58" t="n">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="I36" s="57" t="n"/>
       <c r="J36" s="58" t="n">
@@ -3986,22 +3986,22 @@
       </c>
       <c r="B38" s="57" t="n"/>
       <c r="C38" s="58" t="n">
-        <v>29285</v>
+        <v>30309</v>
       </c>
       <c r="D38" s="58" t="n">
-        <v>32137</v>
+        <v>33263</v>
       </c>
       <c r="E38" s="58" t="n">
-        <v>34101</v>
+        <v>35144</v>
       </c>
       <c r="F38" s="58" t="n">
-        <v>29804</v>
+        <v>30970</v>
       </c>
       <c r="G38" s="58" t="n">
-        <v>23890</v>
+        <v>25226</v>
       </c>
       <c r="H38" s="58" t="n">
-        <v>-5914</v>
+        <v>-5744</v>
       </c>
       <c r="I38" s="57" t="n"/>
       <c r="J38" s="58" t="n">
@@ -4017,10 +4017,10 @@
         <v>34997</v>
       </c>
       <c r="N38" s="57" t="n">
-        <v>23890</v>
+        <v>25226</v>
       </c>
       <c r="O38" s="57" t="n">
-        <v>-11107</v>
+        <v>-9771</v>
       </c>
       <c r="P38" s="57" t="n"/>
       <c r="Q38" s="57" t="n"/>
@@ -4041,22 +4041,22 @@
         </is>
       </c>
       <c r="C39" s="58" t="n">
-        <v>23900</v>
+        <v>24716</v>
       </c>
       <c r="D39" s="58" t="n">
-        <v>26743</v>
+        <v>27706</v>
       </c>
       <c r="E39" s="58" t="n">
-        <v>29092</v>
+        <v>29956</v>
       </c>
       <c r="F39" s="58" t="n">
-        <v>23106</v>
+        <v>24056</v>
       </c>
       <c r="G39" s="58" t="n">
-        <v>19207</v>
+        <v>20372</v>
       </c>
       <c r="H39" s="58" t="n">
-        <v>-3899</v>
+        <v>-3684</v>
       </c>
       <c r="I39" s="57" t="n"/>
       <c r="J39" s="58" t="n">
@@ -4072,10 +4072,10 @@
         <v>27509</v>
       </c>
       <c r="N39" s="57" t="n">
-        <v>19207</v>
+        <v>20372</v>
       </c>
       <c r="O39" s="57" t="n">
-        <v>-8302</v>
+        <v>-7137</v>
       </c>
       <c r="P39" s="57" t="n"/>
       <c r="Q39" s="57" t="n"/>
@@ -4096,22 +4096,22 @@
         </is>
       </c>
       <c r="C40" s="58" t="n">
-        <v>3100</v>
+        <v>3218</v>
       </c>
       <c r="D40" s="58" t="n">
-        <v>3358</v>
+        <v>3465</v>
       </c>
       <c r="E40" s="58" t="n">
-        <v>3871</v>
+        <v>4006</v>
       </c>
       <c r="F40" s="58" t="n">
-        <v>3988</v>
+        <v>4118</v>
       </c>
       <c r="G40" s="58" t="n">
-        <v>3024</v>
+        <v>3161</v>
       </c>
       <c r="H40" s="58" t="n">
-        <v>-964</v>
+        <v>-957</v>
       </c>
       <c r="I40" s="57" t="n"/>
       <c r="J40" s="58" t="n">
@@ -4127,10 +4127,10 @@
         <v>4512</v>
       </c>
       <c r="N40" s="57" t="n">
-        <v>3024</v>
+        <v>3161</v>
       </c>
       <c r="O40" s="57" t="n">
-        <v>-1488</v>
+        <v>-1351</v>
       </c>
       <c r="P40" s="57" t="n"/>
       <c r="Q40" s="57" t="n"/>
@@ -4151,22 +4151,22 @@
         </is>
       </c>
       <c r="C41" s="58" t="n">
-        <v>890</v>
+        <v>936</v>
       </c>
       <c r="D41" s="58" t="n">
-        <v>1096</v>
+        <v>1127</v>
       </c>
       <c r="E41" s="58" t="n">
-        <v>860</v>
+        <v>894</v>
       </c>
       <c r="F41" s="58" t="n">
-        <v>865</v>
+        <v>926</v>
       </c>
       <c r="G41" s="58" t="n">
-        <v>749</v>
+        <v>776</v>
       </c>
       <c r="H41" s="58" t="n">
-        <v>-116</v>
+        <v>-150</v>
       </c>
       <c r="I41" s="57" t="n"/>
       <c r="J41" s="58" t="n">
@@ -4182,10 +4182,10 @@
         <v>1022</v>
       </c>
       <c r="N41" s="57" t="n">
-        <v>749</v>
+        <v>776</v>
       </c>
       <c r="O41" s="57" t="n">
-        <v>-273</v>
+        <v>-246</v>
       </c>
       <c r="P41" s="57" t="n"/>
       <c r="Q41" s="57" t="n"/>
@@ -4206,22 +4206,22 @@
         </is>
       </c>
       <c r="C42" s="58" t="n">
-        <v>1321</v>
+        <v>1364</v>
       </c>
       <c r="D42" s="58" t="n">
-        <v>782</v>
+        <v>800</v>
       </c>
       <c r="E42" s="58" t="n">
-        <v>245</v>
+        <v>251</v>
       </c>
       <c r="F42" s="58" t="n">
-        <v>213</v>
+        <v>218</v>
       </c>
       <c r="G42" s="58" t="n">
-        <v>182</v>
+        <v>188</v>
       </c>
       <c r="H42" s="58" t="n">
-        <v>-31</v>
+        <v>-30</v>
       </c>
       <c r="I42" s="57" t="n"/>
       <c r="J42" s="58" t="n">
@@ -4237,10 +4237,10 @@
         <v>246</v>
       </c>
       <c r="N42" s="57" t="n">
-        <v>182</v>
+        <v>188</v>
       </c>
       <c r="O42" s="57" t="n">
-        <v>-64</v>
+        <v>-58</v>
       </c>
       <c r="P42" s="57" t="n"/>
       <c r="Q42" s="57" t="n"/>
@@ -4261,22 +4261,22 @@
         </is>
       </c>
       <c r="C43" s="58" t="n">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="D43" s="58" t="n">
-        <v>158</v>
+        <v>165</v>
       </c>
       <c r="E43" s="58" t="n">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="F43" s="58" t="n">
-        <v>1632</v>
+        <v>1652</v>
       </c>
       <c r="G43" s="58" t="n">
-        <v>728</v>
+        <v>729</v>
       </c>
       <c r="H43" s="58" t="n">
-        <v>-904</v>
+        <v>-923</v>
       </c>
       <c r="I43" s="57" t="n"/>
       <c r="J43" s="58" t="n">
@@ -4292,10 +4292,10 @@
         <v>1708</v>
       </c>
       <c r="N43" s="57" t="n">
-        <v>728</v>
+        <v>729</v>
       </c>
       <c r="O43" s="57" t="n">
-        <v>-980</v>
+        <v>-979</v>
       </c>
       <c r="P43" s="57" t="n"/>
       <c r="Q43" s="57" t="n"/>
@@ -4343,22 +4343,22 @@
       </c>
       <c r="B45" s="57" t="n"/>
       <c r="C45" s="58" t="n">
-        <v>2123</v>
+        <v>2186</v>
       </c>
       <c r="D45" s="58" t="n">
-        <v>2847</v>
+        <v>2968</v>
       </c>
       <c r="E45" s="58" t="n">
-        <v>3796</v>
+        <v>3911</v>
       </c>
       <c r="F45" s="58" t="n">
-        <v>2661</v>
+        <v>2770</v>
       </c>
       <c r="G45" s="58" t="n">
-        <v>1713</v>
+        <v>1827</v>
       </c>
       <c r="H45" s="58" t="n">
-        <v>-948</v>
+        <v>-943</v>
       </c>
       <c r="I45" s="57" t="n"/>
       <c r="J45" s="58" t="n">
@@ -4374,10 +4374,10 @@
         <v>3136</v>
       </c>
       <c r="N45" s="57" t="n">
-        <v>1713</v>
+        <v>1827</v>
       </c>
       <c r="O45" s="57" t="n">
-        <v>-1423</v>
+        <v>-1309</v>
       </c>
       <c r="P45" s="57" t="n"/>
       <c r="Q45" s="57" t="n"/>
@@ -4398,22 +4398,22 @@
         </is>
       </c>
       <c r="C46" s="58" t="n">
-        <v>1735</v>
+        <v>1788</v>
       </c>
       <c r="D46" s="58" t="n">
-        <v>2443</v>
+        <v>2542</v>
       </c>
       <c r="E46" s="58" t="n">
-        <v>3341</v>
+        <v>3441</v>
       </c>
       <c r="F46" s="58" t="n">
-        <v>2365</v>
+        <v>2469</v>
       </c>
       <c r="G46" s="58" t="n">
-        <v>1511</v>
+        <v>1617</v>
       </c>
       <c r="H46" s="58" t="n">
-        <v>-854</v>
+        <v>-852</v>
       </c>
       <c r="I46" s="57" t="n"/>
       <c r="J46" s="58" t="n">
@@ -4429,10 +4429,10 @@
         <v>2798</v>
       </c>
       <c r="N46" s="57" t="n">
-        <v>1511</v>
+        <v>1617</v>
       </c>
       <c r="O46" s="57" t="n">
-        <v>-1287</v>
+        <v>-1181</v>
       </c>
       <c r="P46" s="57" t="n"/>
       <c r="Q46" s="57" t="n"/>
@@ -4453,22 +4453,22 @@
         </is>
       </c>
       <c r="C47" s="58" t="n">
-        <v>158</v>
+        <v>164</v>
       </c>
       <c r="D47" s="58" t="n">
-        <v>245</v>
+        <v>257</v>
       </c>
       <c r="E47" s="58" t="n">
-        <v>247</v>
+        <v>254</v>
       </c>
       <c r="F47" s="58" t="n">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="G47" s="58" t="n">
-        <v>109</v>
+        <v>114</v>
       </c>
       <c r="H47" s="58" t="n">
-        <v>-52</v>
+        <v>-49</v>
       </c>
       <c r="I47" s="57" t="n"/>
       <c r="J47" s="58" t="n">
@@ -4484,10 +4484,10 @@
         <v>178</v>
       </c>
       <c r="N47" s="57" t="n">
-        <v>109</v>
+        <v>114</v>
       </c>
       <c r="O47" s="57" t="n">
-        <v>-69</v>
+        <v>-64</v>
       </c>
       <c r="P47" s="57" t="n"/>
       <c r="Q47" s="57" t="n"/>
@@ -4508,19 +4508,19 @@
         </is>
       </c>
       <c r="C48" s="58" t="n">
-        <v>211</v>
+        <v>215</v>
       </c>
       <c r="D48" s="58" t="n">
-        <v>137</v>
+        <v>146</v>
       </c>
       <c r="E48" s="58" t="n">
-        <v>204</v>
+        <v>212</v>
       </c>
       <c r="F48" s="58" t="n">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="G48" s="58" t="n">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="H48" s="58" t="n">
         <v>-30</v>
@@ -4539,10 +4539,10 @@
         <v>106</v>
       </c>
       <c r="N48" s="57" t="n">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="O48" s="57" t="n">
-        <v>-46</v>
+        <v>-43</v>
       </c>
       <c r="P48" s="57" t="n"/>
       <c r="Q48" s="57" t="n"/>
@@ -4566,7 +4566,7 @@
         <v>19</v>
       </c>
       <c r="D49" s="58" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E49" s="58" t="n">
         <v>3</v>
@@ -4712,10 +4712,10 @@
         <v>79</v>
       </c>
       <c r="G52" s="58" t="n">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="H52" s="58" t="n">
-        <v>-11</v>
+        <v>-9</v>
       </c>
       <c r="I52" s="57" t="n"/>
       <c r="J52" s="58" t="n">
@@ -4731,10 +4731,10 @@
         <v>0</v>
       </c>
       <c r="N52" s="57" t="n">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="O52" s="57" t="n">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="P52" s="57" t="n"/>
       <c r="Q52" s="57" t="n"/>
@@ -4755,22 +4755,22 @@
         </is>
       </c>
       <c r="C53" s="58" t="n">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="D53" s="58" t="n">
         <v>189</v>
       </c>
       <c r="E53" s="58" t="n">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="F53" s="58" t="n">
         <v>77</v>
       </c>
       <c r="G53" s="58" t="n">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="H53" s="58" t="n">
-        <v>-16</v>
+        <v>-14</v>
       </c>
       <c r="I53" s="57" t="n"/>
       <c r="J53" s="58" t="n">
@@ -4786,10 +4786,10 @@
         <v>88</v>
       </c>
       <c r="N53" s="57" t="n">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="O53" s="57" t="n">
-        <v>-27</v>
+        <v>-25</v>
       </c>
       <c r="P53" s="57" t="n"/>
       <c r="Q53" s="57" t="n"/>
@@ -4920,7 +4920,7 @@
         </is>
       </c>
       <c r="C56" s="58" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D56" s="58" t="n">
         <v>2</v>

</xml_diff>

<commit_message>
docs(hubs): update hub BRDs, vehicle deductible page PRD, meeting recaps, and October MTD tracking
</commit_message>
<xml_diff>
--- a/05_HUBS/cinema/cinema-hub-roadmap.xlsx
+++ b/05_HUBS/cinema/cinema-hub-roadmap.xlsx
@@ -1,24 +1,24 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Readme" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Performance" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Roadmap" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Market Sizing &amp; Opportunities" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Content Structure" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KPIs &amp; Target Metrics" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resources" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Utilities &amp; Formula Specs" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Subpages Directory" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Event Tracking Flow" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bộ Param Master Registry" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracking Class &amp; HTML Specs" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="Readme" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Performance" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Roadmap" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Market Sizing &amp; Opportunities" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Content Structure" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="KPIs &amp; Target Metrics" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Resources" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Utilities &amp; Formula Specs" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Subpages Directory" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Event Tracking Flow" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Bộ Param Master Registry" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Tracking Class &amp; HTML Specs" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -2430,7 +2430,7 @@
     <row r="1">
       <c r="A1" s="6" t="inlineStr">
         <is>
-          <t>BÁO CÁO PHÂN TÍCH HIỆU SUẤT VẬN HÀNH &amp; TRAFFIC - CINEMA HUB (MTD 27D - CẮT NGÀY 27/09/2026)</t>
+          <t>BÁO CÁO PHÂN TÍCH HIỆU SUẤT VẬN HÀNH &amp; TRAFFIC - CINEMA HUB (FULL MONTH THÁNG 9/2026 - CHỐT SỔ 30 NGÀY)</t>
         </is>
       </c>
     </row>
@@ -2447,14 +2447,34 @@
           <t>Thông Số Dashboard Hub</t>
         </is>
       </c>
-      <c r="B4" s="43" t="n"/>
-      <c r="C4" s="43" t="n"/>
-      <c r="D4" s="43" t="n"/>
-      <c r="E4" s="43" t="n"/>
-      <c r="F4" s="37" t="n"/>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Phân Loại Zone</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Số Thực Tế Full Month T9</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Nhịp Độ Ngày (Daily Pace)</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Actual 30d</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Target Tháng 9</t>
+        </is>
+      </c>
       <c r="G4" s="50" t="inlineStr">
         <is>
-          <t>Tỷ Lệ % Projected</t>
+          <t>Tỷ Lệ % Hoàn Thành</t>
         </is>
       </c>
       <c r="H4" s="50" t="inlineStr">
@@ -2475,23 +2495,23 @@
         </is>
       </c>
       <c r="C5" s="52" t="n">
-        <v>1086874</v>
+        <v>1220075</v>
       </c>
       <c r="D5" s="52" t="n">
-        <v>40254.6</v>
+        <v>40669.2</v>
       </c>
       <c r="E5" s="52" t="n">
-        <v>1207637.8</v>
+        <v>1220075</v>
       </c>
       <c r="F5" s="52" t="n">
         <v>964394</v>
       </c>
       <c r="G5" s="53" t="n">
-        <v>1.127</v>
+        <v>1.2651</v>
       </c>
       <c r="H5" s="51" t="inlineStr">
         <is>
-          <t>VƯỢT TARGET THÁNG 9 +12.7% TRƯỚC HẠN (112.7% MTD, Forecast trọn tháng 1.2M - 125.2%)</t>
+          <t>VƯỢT TARGET THÁNG 9 +26.5% CHÍNH THỨC (CÁN MỐC KỶ LỤC LỊCH SỬ &gt;1.22M PVS)</t>
         </is>
       </c>
     </row>
@@ -2640,7 +2660,7 @@
         <v>699471</v>
       </c>
       <c r="G11" s="58" t="n">
-        <v>1086874</v>
+        <v>1220075</v>
       </c>
       <c r="H11" s="58" t="n">
         <v>387403</v>
@@ -30830,12 +30850,11 @@
       <c r="Y1017" s="57" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="8">
+  <mergeCells count="7">
     <mergeCell ref="B25:I25"/>
     <mergeCell ref="B24:I24"/>
     <mergeCell ref="A14:I14"/>
     <mergeCell ref="B22:I22"/>
-    <mergeCell ref="A4:F4"/>
     <mergeCell ref="B23:I23"/>
     <mergeCell ref="A21:I21"/>
     <mergeCell ref="B26:I26"/>

</xml_diff>